<commit_message>
Solved some file upload and export related issues
</commit_message>
<xml_diff>
--- a/Command-Center-Backend/Templates/DixonDailyReportTemplate.xlsx
+++ b/Command-Center-Backend/Templates/DixonDailyReportTemplate.xlsx
@@ -2851,49 +2851,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>291353</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>1</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>30</xdr:col>
-      <xdr:colOff>3315838</xdr:colOff>
-      <xdr:row>42</xdr:row>
-      <xdr:rowOff>10595</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="17638059" y="8594913"/>
-          <a:ext cx="7394779" cy="2520711"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -5089,7 +5046,6 @@
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="29" orientation="landscape" r:id="rId1"/>
-  <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>

</xml_diff>